<commit_message>
Expand episode system with chapters, cutscene commands, and visual JSON editor.
Add multi-chapter episodes with unlock progress, combat tablero field, full card previews, auto-advance for scene/fade commands, and crearEpisodios.html editor API. Includes episodio2 assets and CONTEXT.md documentation.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/episodios.xlsx
+++ b/public/resources/episodios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D44AAE39-764B-44F8-AEAE-C98739010C95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3D40552-2EE0-4E2D-8C50-49B07F93EB92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7200" yWindow="4215" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -48,9 +48,6 @@
     <t>Sigue a una Supergirl desilusionada que viaja al espacio para escapar de su pasado. Allí se cruza con Ruthye, una niña alienígena que busca venganza contra un mercenario que asesinó a su padre. Ambas, junto al Superperro Krypto, se embarcan en una épica cacería intergaláctica al estilo del western.</t>
   </si>
   <si>
-    <t>episodio1.json</t>
-  </si>
-  <si>
     <t>https://i.ibb.co/Y4hSWkyS/Supergirl-Wo-T.jpg</t>
   </si>
   <si>
@@ -64,6 +61,9 @@
   </si>
   <si>
     <t>episodio2.json</t>
+  </si>
+  <si>
+    <t>ejemplo.json</t>
   </si>
 </sst>
 </file>
@@ -440,10 +440,10 @@
         <v>6</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -456,16 +456,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add internal card editor and dev-branch Git push for content tools.
Enable crearEpisodios and editarCartas on Render dev via RENDER_GIT_BRANCH, with optional commit+push to GitHub from each editor toolbar.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/episodios.xlsx
+++ b/public/resources/episodios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3D40552-2EE0-4E2D-8C50-49B07F93EB92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{881A0B57-2A11-44A1-95C0-F7FD6C041D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7200" yWindow="4215" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -468,6 +468,13 @@
         <v>11</v>
       </c>
     </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Improve episodes carousel UI and required-cards 3D panel.
Enlarge episode panels, reuse evento-enemigos-carrusel for required cards with collection badge, and update episodio sample content.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/resources/episodios.xlsx
+++ b/public/resources/episodios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\DC Battle Cards\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{881A0B57-2A11-44A1-95C0-F7FD6C041D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CE8E46E-5C10-41FA-BA42-50C0AE936885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7200" yWindow="4215" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>evento_id</t>
   </si>
@@ -40,30 +40,6 @@
   </si>
   <si>
     <t>imagen</t>
-  </si>
-  <si>
-    <t>Supergirl: Woman of Tomorrow</t>
-  </si>
-  <si>
-    <t>Sigue a una Supergirl desilusionada que viaja al espacio para escapar de su pasado. Allí se cruza con Ruthye, una niña alienígena que busca venganza contra un mercenario que asesinó a su padre. Ambas, junto al Superperro Krypto, se embarcan en una épica cacería intergaláctica al estilo del western.</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/Y4hSWkyS/Supergirl-Wo-T.jpg</t>
-  </si>
-  <si>
-    <t>Aves de Presa</t>
-  </si>
-  <si>
-    <t>Ponte en la piel de las Heroinas más cañeras e imparables de todas, donde se enfrentarán a una serie de desafios que las podrán a prueba de formas inimaginables.</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/7dPzn7FG/bop.jpg</t>
-  </si>
-  <si>
-    <t>episodio2.json</t>
-  </si>
-  <si>
-    <t>ejemplo.json</t>
   </si>
 </sst>
 </file>
@@ -430,21 +406,11 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -452,21 +418,11 @@
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>

</xml_diff>